<commit_message>
new commit in login branch
</commit_message>
<xml_diff>
--- a/TestData/loginData.xlsx
+++ b/TestData/loginData.xlsx
@@ -1,45 +1,88 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\expleo company traning doc\Python-DWS\PYTHON_DEMOWEBSHOP\TestData\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5367C91F-9587-4D29-A980-16BEE035A0AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView tabRatio="500"/>
+    <workbookView xWindow="3432" yWindow="1908" windowWidth="17280" windowHeight="8880" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet r:id="rId1" name="Sheet1" sheetId="1"/>
+    <sheet name="login" sheetId="1" r:id="rId1"/>
+    <sheet name="recovery" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="0" iterate="1" iterateCount="1000" iterateDelta="0.01"/>
 </workbook>
 </file>
 
-<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
-  <metadataTypes count="1">
-    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
-  </metadataTypes>
-  <futureMetadata name="XLDAPR" count="1">
-    <bk>
-      <extLst>
-        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
-          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
-        </ext>
-      </extLst>
-    </bk>
-  </futureMetadata>
-  <cellMetadata count="1">
-    <bk>
-      <rc t="1" v="0"/>
-    </bk>
-  </cellMetadata>
-</metadata>
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="15">
+  <si>
+    <t>email</t>
+  </si>
+  <si>
+    <t>password</t>
+  </si>
+  <si>
+    <t>error_message</t>
+  </si>
+  <si>
+    <t>haritha@gmail.com</t>
+  </si>
+  <si>
+    <t>haritha</t>
+  </si>
+  <si>
+    <t>The credentials provided are incorrect</t>
+  </si>
+  <si>
+    <t>haritha11@gmail.com</t>
+  </si>
+  <si>
+    <t>hari</t>
+  </si>
+  <si>
+    <t>No customer account found</t>
+  </si>
+  <si>
+    <t>Login was unsuccessful. Please correct the errors and try again.</t>
+  </si>
+  <si>
+    <t>message</t>
+  </si>
+  <si>
+    <t>Email with instructions has been sent to you.</t>
+  </si>
+  <si>
+    <t>Wrong email</t>
+  </si>
+  <si>
+    <t>harithagmail.com</t>
+  </si>
+  <si>
+    <t>Enter your email</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <scheme val="minor"/>
     </font>
@@ -58,37 +101,49 @@
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
     </border>
     <border>
-      <left>
-        <color rgb="FF000000"/>
-      </left>
-      <right>
-        <color rgb="FF000000"/>
-      </right>
-      <top>
-        <color rgb="FF000000"/>
-      </top>
-      <bottom>
-        <color rgb="FF000000"/>
-      </bottom>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1">
-      <alignment horizontal="general" vertical="top"/>
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="top"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0">
       <alignment vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1">
+      <alignment vertical="top"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0"/>
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -400,17 +455,121 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{AD60C143-597E-41FB-B2FD-E8EA9569F403}" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1:T200"/>
-  <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
-  <sheetData/>
-  <printOptions/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AD60C143-597E-41FB-B2FD-E8EA9569F403}">
+  <dimension ref="A1:C6"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="19.21875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.77734375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="32.33203125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C4" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B5" t="s">
+        <v>4</v>
+      </c>
+      <c r="C5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="1" orientation="portrait"/>
+  <pageSetup orientation="portrait"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;C&amp;R</oddHeader>
     <oddFooter>&amp;L&amp;C&amp;R</oddFooter>
   </headerFooter>
-  <extLst/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7BB86CF5-BCD3-4DCB-8F43-4BFF43B257CF}">
+  <dimension ref="A1:B4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="37.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.44140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B3" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A2" r:id="rId1" xr:uid="{3D650744-8032-4ABB-9F1C-F0B014C37DA5}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>